<commit_message>
Sprememba excel file-a za naloge + dodana powerpoint predstavitev
</commit_message>
<xml_diff>
--- a/DanielGrozdanovic/projektnaNaloga/DanielGrozdanovic.xlsx
+++ b/DanielGrozdanovic/projektnaNaloga/DanielGrozdanovic.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grozd\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grozd\Documents\naloge_ro\DanielGrozdanovic\projektnaNaloga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA671E3-28AA-4CCE-8FCD-BCD2D8B09FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5846D9-786B-41E3-873D-8165BD06850C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -398,12 +398,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -651,79 +659,79 @@
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1505,44 +1513,44 @@
       <c r="C2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="23" t="s">
+      <c r="G2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="H2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="M2" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="N2" s="22" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" spans="2:16" ht="201.6" x14ac:dyDescent="0.3">
       <c r="B3" s="11"/>
       <c r="C3" s="12"/>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="26" t="s">
         <v>57</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -1575,7 +1583,7 @@
       <c r="N3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="18" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1586,10 +1594,10 @@
       <c r="C4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>47</v>
       </c>
       <c r="F4" s="4"/>
@@ -1601,7 +1609,7 @@
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-      <c r="P4" s="20" t="s">
+      <c r="P4" s="19" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1612,32 +1620,32 @@
       <c r="C5" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="23" t="s">
+      <c r="J5" s="22" t="s">
         <v>18</v>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="15"/>
-      <c r="P5" s="21" t="s">
+      <c r="P5" s="20" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1675,16 +1683,16 @@
       <c r="C7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="22" t="s">
         <v>59</v>
       </c>
       <c r="H7" s="4"/>
@@ -1723,22 +1731,22 @@
       <c r="C9" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="22" t="s">
         <v>26</v>
       </c>
       <c r="J9" s="4"/>
@@ -1781,10 +1789,10 @@
       <c r="C11" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="22" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="4"/>
@@ -1823,16 +1831,16 @@
       <c r="C13" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="22" t="s">
         <v>30</v>
       </c>
       <c r="H13" s="4"/>
@@ -1869,16 +1877,16 @@
       <c r="C15" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="23" t="s">
+      <c r="G15" s="22" t="s">
         <v>32</v>
       </c>
       <c r="H15" s="4"/>
@@ -1919,10 +1927,10 @@
       <c r="C17" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="22" t="s">
         <v>78</v>
       </c>
       <c r="F17" s="4"/>
@@ -1957,19 +1965,19 @@
       <c r="C19" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="G19" s="23" t="s">
+      <c r="G19" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" s="22" t="s">
         <v>93</v>
       </c>
       <c r="I19" s="4"/>
@@ -2007,10 +2015,10 @@
       <c r="C21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="22" t="s">
         <v>95</v>
       </c>
       <c r="F21" s="4"/>
@@ -2026,7 +2034,7 @@
     <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" s="9"/>
       <c r="C22" s="10"/>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="23" t="s">
         <v>94</v>
       </c>
       <c r="E22" s="4"/>
@@ -2047,19 +2055,19 @@
       <c r="C23" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="25" t="s">
+      <c r="D23" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G23" s="26" t="s">
+      <c r="G23" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="26" t="s">
+      <c r="H23" s="22" t="s">
         <v>96</v>
       </c>
       <c r="I23" s="4"/>
@@ -2076,7 +2084,7 @@
       <c r="C24" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="25" t="s">
         <v>40</v>
       </c>
       <c r="E24" s="4"/>
@@ -2097,7 +2105,7 @@
       <c r="C25" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D25" s="27" t="s">
+      <c r="D25" s="25" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="4"/>
@@ -2112,13 +2120,13 @@
       <c r="N25" s="15"/>
     </row>
     <row r="26" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="17">
+      <c r="B26" s="16">
         <v>9</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="16" t="s">
+      <c r="C26" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="27" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>